<commit_message>
Enhance .gitignore, update README for development instructions, and refactor settings.py for dynamic project root resolution
</commit_message>
<xml_diff>
--- a/data/db/documents.xlsx
+++ b/data/db/documents.xlsx
@@ -33040,7 +33040,7 @@
       </c>
       <c r="E1048" s="2" t="inlineStr">
         <is>
-          <t>DOWNLOADED</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1048" s="2" t="inlineStr">
@@ -33072,7 +33072,7 @@
       </c>
       <c r="E1049" s="2" t="inlineStr">
         <is>
-          <t>DOWNLOADED</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1049" s="2" t="inlineStr">
@@ -33104,7 +33104,7 @@
       </c>
       <c r="E1050" s="2" t="inlineStr">
         <is>
-          <t>DOWNLOADED</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1050" s="2" t="inlineStr">
@@ -33136,7 +33136,7 @@
       </c>
       <c r="E1051" s="2" t="inlineStr">
         <is>
-          <t>DOWNLOADED</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1051" s="2" t="inlineStr">
@@ -33168,7 +33168,7 @@
       </c>
       <c r="E1052" s="2" t="inlineStr">
         <is>
-          <t>DOWNLOADED</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1052" s="2" t="inlineStr">
@@ -33200,7 +33200,7 @@
       </c>
       <c r="E1053" s="2" t="inlineStr">
         <is>
-          <t>DOWNLOADED</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1053" s="2" t="inlineStr">
@@ -33220,7 +33220,11 @@
           <t>PR2ME-PIL-QTY-59-HOP-3420-13-02</t>
         </is>
       </c>
-      <c r="C1054" s="2" t="inlineStr"/>
+      <c r="C1054" s="2" t="inlineStr">
+        <is>
+          <t>Mechanical HOP of Subsystem 3420-13-02 3422-FC-067 3422-FC-067-M01 2nd Oxide Cleaner Cell 2</t>
+        </is>
+      </c>
       <c r="D1054" s="2" t="inlineStr">
         <is>
           <t>Mechanical</t>
@@ -33228,7 +33232,7 @@
       </c>
       <c r="E1054" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1054" s="2" t="inlineStr">
@@ -33248,7 +33252,11 @@
           <t>PR2ME-PIL-QTY-50-HOP-FT-3420-13-02</t>
         </is>
       </c>
-      <c r="C1055" s="2" t="inlineStr"/>
+      <c r="C1055" s="2" t="inlineStr">
+        <is>
+          <t>Piping HOP of 2nd Oxide Cleaner Cell 2 &amp; Agitator</t>
+        </is>
+      </c>
       <c r="D1055" s="2" t="inlineStr">
         <is>
           <t>Piping</t>
@@ -33256,7 +33264,7 @@
       </c>
       <c r="E1055" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1055" s="2" t="inlineStr">
@@ -33276,15 +33284,19 @@
           <t>PR2ME-PIL-QTY-70-HOP-3420-13-02</t>
         </is>
       </c>
-      <c r="C1056" s="2" t="inlineStr"/>
+      <c r="C1056" s="2" t="inlineStr">
+        <is>
+          <t>Instrument HOP of Subsystem 3420-13-02 2nd Oxide Cleaner Cell 2 &amp; Agitator</t>
+        </is>
+      </c>
       <c r="D1056" s="2" t="inlineStr">
         <is>
-          <t>No Discipline</t>
+          <t>Telecommunication</t>
         </is>
       </c>
       <c r="E1056" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1056" s="2" t="inlineStr">
@@ -33304,15 +33316,19 @@
           <t>PR2ME-PIL-QTY-65-HOP-3420-13-02</t>
         </is>
       </c>
-      <c r="C1057" s="2" t="inlineStr"/>
+      <c r="C1057" s="2" t="inlineStr">
+        <is>
+          <t>Electrical HOP of Subsystem 3420-13-02 2nd Oxide Cleaner Cell 2 &amp; Agitator</t>
+        </is>
+      </c>
       <c r="D1057" s="2" t="inlineStr">
         <is>
-          <t>No Discipline</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="E1057" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1057" s="2" t="inlineStr">
@@ -33332,7 +33348,11 @@
           <t>PR2ME-PIL-QTY-59-HOP-3140-01-01</t>
         </is>
       </c>
-      <c r="C1058" s="2" t="inlineStr"/>
+      <c r="C1058" s="2" t="inlineStr">
+        <is>
+          <t>Mechanical HOP of Subsystem 3140-01-01 3141-CV-007, 3141-BS-007, 3141-BS-008, 3141-BS-010, 3141-CH-009 SAG Mill Pebble Screen Oversize Conveyor 1</t>
+        </is>
+      </c>
       <c r="D1058" s="2" t="inlineStr">
         <is>
           <t>Mechanical</t>
@@ -33340,7 +33360,7 @@
       </c>
       <c r="E1058" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1058" s="2" t="inlineStr">
@@ -33360,15 +33380,19 @@
           <t>PR2ME-PIL-QTY-70-HOP-3140-01-01</t>
         </is>
       </c>
-      <c r="C1059" s="2" t="inlineStr"/>
+      <c r="C1059" s="2" t="inlineStr">
+        <is>
+          <t>Instrument HOP of Subsystem 3140-01-01 SAG Mill Pebble Screen Oversize Conveyor 1</t>
+        </is>
+      </c>
       <c r="D1059" s="2" t="inlineStr">
         <is>
-          <t>No Discipline</t>
+          <t>Telecommunication</t>
         </is>
       </c>
       <c r="E1059" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1059" s="2" t="inlineStr">
@@ -33388,15 +33412,19 @@
           <t>PR2ME-PIL-QTY-65-HOP-3140-01-01</t>
         </is>
       </c>
-      <c r="C1060" s="2" t="inlineStr"/>
+      <c r="C1060" s="2" t="inlineStr">
+        <is>
+          <t>Electrical HOP of Subsystem 3140-01-01 SAG Mill Pebble Screen Oversize Conveyor 1</t>
+        </is>
+      </c>
       <c r="D1060" s="2" t="inlineStr">
         <is>
-          <t>No Discipline</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="E1060" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1060" s="2" t="inlineStr">
@@ -33416,7 +33444,11 @@
           <t>PR2ME-PIL-QTY-59-HOP-3220-07-02</t>
         </is>
       </c>
-      <c r="C1061" s="2" t="inlineStr"/>
+      <c r="C1061" s="2" t="inlineStr">
+        <is>
+          <t>Mechanical HOP of Subsystem 3220-07-02 3223-SC-404 Ball Mill 6 Crushed Pebble Conveyor Weightometer</t>
+        </is>
+      </c>
       <c r="D1061" s="2" t="inlineStr">
         <is>
           <t>Mechanical</t>
@@ -33424,7 +33456,7 @@
       </c>
       <c r="E1061" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1061" s="2" t="inlineStr">
@@ -33444,15 +33476,19 @@
           <t>PR2ME-PIL-QTY-70-HOP-3220-07-02</t>
         </is>
       </c>
-      <c r="C1062" s="2" t="inlineStr"/>
+      <c r="C1062" s="2" t="inlineStr">
+        <is>
+          <t>Instrument HOP of Subsystem 3220-07-02 Ball Mill 6 Crushed Pebble Conveyor Weightometer</t>
+        </is>
+      </c>
       <c r="D1062" s="2" t="inlineStr">
         <is>
-          <t>No Discipline</t>
+          <t>Telecommunication</t>
         </is>
       </c>
       <c r="E1062" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1062" s="2" t="inlineStr">
@@ -33472,7 +33508,11 @@
           <t>PR2ME-PIL-QTY-59-HOP-3580-05-01</t>
         </is>
       </c>
-      <c r="C1063" s="2" t="inlineStr"/>
+      <c r="C1063" s="2" t="inlineStr">
+        <is>
+          <t>Mechanical HOP of Lime Slacking Mill 1 Cyclone Feed Pump 1 &amp; VSD 3580-05-01</t>
+        </is>
+      </c>
       <c r="D1063" s="2" t="inlineStr">
         <is>
           <t>Mechanical</t>
@@ -33480,7 +33520,7 @@
       </c>
       <c r="E1063" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1063" s="2" t="inlineStr">
@@ -33500,7 +33540,11 @@
           <t>PR2ME-PIL-QTY-50-HOP-GWF-3580-05-01</t>
         </is>
       </c>
-      <c r="C1064" s="2" t="inlineStr"/>
+      <c r="C1064" s="2" t="inlineStr">
+        <is>
+          <t>Piping HOP of Lime Slacking Mill 1 Cyclone Feed Pump 1 &amp; VSD</t>
+        </is>
+      </c>
       <c r="D1064" s="2" t="inlineStr">
         <is>
           <t>Piping</t>
@@ -33508,7 +33552,7 @@
       </c>
       <c r="E1064" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1064" s="2" t="inlineStr">
@@ -33528,15 +33572,19 @@
           <t>PR2ME-PIL-QTY-70-HOP-3580-05-01</t>
         </is>
       </c>
-      <c r="C1065" s="2" t="inlineStr"/>
+      <c r="C1065" s="2" t="inlineStr">
+        <is>
+          <t>Instrument HOP of Subsystem 3580-05-01 Lime Slaking Mill 1 Cyclone Feed Pump 1 &amp; VSD</t>
+        </is>
+      </c>
       <c r="D1065" s="2" t="inlineStr">
         <is>
-          <t>No Discipline</t>
+          <t>Telecommunication</t>
         </is>
       </c>
       <c r="E1065" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1065" s="2" t="inlineStr">
@@ -33556,15 +33604,19 @@
           <t>PR2ME-PIL-QTY-65-HOP-3580-05-01</t>
         </is>
       </c>
-      <c r="C1066" s="2" t="inlineStr"/>
+      <c r="C1066" s="2" t="inlineStr">
+        <is>
+          <t>Electrical HOP of Subsystem 3580-05-01 Lime Slaking Mill 1 Cyclone Feed Pump 1 &amp; VSD</t>
+        </is>
+      </c>
       <c r="D1066" s="2" t="inlineStr">
         <is>
-          <t>No Discipline</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="E1066" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1066" s="2" t="inlineStr">
@@ -33584,7 +33636,11 @@
           <t>PR2ME-PIL-QTY-59-HOP-3580-07-03</t>
         </is>
       </c>
-      <c r="C1067" s="2" t="inlineStr"/>
+      <c r="C1067" s="2" t="inlineStr">
+        <is>
+          <t>Mechanical HOP of Lime Transfer Pumps 3 3580-07-03</t>
+        </is>
+      </c>
       <c r="D1067" s="2" t="inlineStr">
         <is>
           <t>Mechanical</t>
@@ -33592,7 +33648,7 @@
       </c>
       <c r="E1067" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1067" s="2" t="inlineStr">
@@ -33612,7 +33668,11 @@
           <t>PR2ME-PIL-QTY-50-HOP-ML-3580-07-03</t>
         </is>
       </c>
-      <c r="C1068" s="2" t="inlineStr"/>
+      <c r="C1068" s="2" t="inlineStr">
+        <is>
+          <t>Piping HOP of Lime Transfer Pump 3</t>
+        </is>
+      </c>
       <c r="D1068" s="2" t="inlineStr">
         <is>
           <t>Piping</t>
@@ -33620,7 +33680,7 @@
       </c>
       <c r="E1068" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1068" s="2" t="inlineStr">
@@ -33640,15 +33700,19 @@
           <t>PR2ME-PIL-QTY-65-HOP-3580-07-03</t>
         </is>
       </c>
-      <c r="C1069" s="2" t="inlineStr"/>
+      <c r="C1069" s="2" t="inlineStr">
+        <is>
+          <t>Electrical HOP of Subsystem 3580-07-03 Lime Transfer Pump 3</t>
+        </is>
+      </c>
       <c r="D1069" s="2" t="inlineStr">
         <is>
-          <t>No Discipline</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="E1069" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1069" s="2" t="inlineStr">
@@ -33668,15 +33732,19 @@
           <t>PR2ME-PIL-QTY-70-HOP-3580-07-03</t>
         </is>
       </c>
-      <c r="C1070" s="2" t="inlineStr"/>
+      <c r="C1070" s="2" t="inlineStr">
+        <is>
+          <t>Instrument HOP of Subsystem 3580-07-03 Lime Transfer Pump 3</t>
+        </is>
+      </c>
       <c r="D1070" s="2" t="inlineStr">
         <is>
-          <t>No Discipline</t>
+          <t>Telecommunication</t>
         </is>
       </c>
       <c r="E1070" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1070" s="2" t="inlineStr">
@@ -33696,15 +33764,19 @@
           <t>PR2ME-PIL-QTY-70-HOP-2191-90-01</t>
         </is>
       </c>
-      <c r="C1071" s="2" t="inlineStr"/>
+      <c r="C1071" s="2" t="inlineStr">
+        <is>
+          <t>Instrument (PCS) HOP of Subsystem 2191-90-01 Camera-Network</t>
+        </is>
+      </c>
       <c r="D1071" s="2" t="inlineStr">
         <is>
-          <t>No Discipline</t>
+          <t>Telecommunication</t>
         </is>
       </c>
       <c r="E1071" s="2" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>UPLOADED_FILE</t>
         </is>
       </c>
       <c r="F1071" s="2" t="inlineStr">

</xml_diff>